<commit_message>
feat: Implement non-overlapping smoke screen strategy
This commit introduces a new strategy for smoke screen deployment where the goal is to maximize total coverage time while minimizing overlap between different UAVs. It includes a differential evolution algorithm to find optimal parameters for each UAV's deployment and detonation timing. The fitness function penalizes overlapping coverage periods. Results are saved to an Excel file.

Co-authored-by: b35etzhangmingyu <b35etzhangmingyu@126.com>
</commit_message>
<xml_diff>
--- a/result2.xlsx
+++ b/result2.xlsx
@@ -502,40 +502,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.9996378528072006</v>
+        <v>-0.9998300494693119</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02691028121386745</v>
+        <v>0.01843562253338214</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>117.6881701853208</v>
+        <v>95.15925128686945</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5064518630431503</v>
+        <v>1.342452273460086</v>
       </c>
       <c r="G2" t="n">
-        <v>3.498939175981285</v>
+        <v>3.436929578649536</v>
       </c>
       <c r="H2" t="n">
-        <v>17740.41819215298</v>
+        <v>17672.27495739769</v>
       </c>
       <c r="I2" t="n">
-        <v>1.603944068235674</v>
+        <v>2.355090922428467</v>
       </c>
       <c r="J2" t="n">
         <v>1800</v>
       </c>
       <c r="K2" t="n">
-        <v>17328.78356927082</v>
+        <v>17345.27489524821</v>
       </c>
       <c r="L2" t="n">
-        <v>12.68516055880359</v>
+        <v>8.384565348987348</v>
       </c>
       <c r="M2" t="n">
-        <v>1740.00525946196</v>
+        <v>1742.112917607415</v>
       </c>
     </row>
     <row r="3">
@@ -545,40 +545,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.9999998662614554</v>
+        <v>-0.7359202316880927</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0005171818550472835</v>
+        <v>0.6770682481051257</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>120.1804064828093</v>
+        <v>94.23055544662384</v>
       </c>
       <c r="F3" t="n">
-        <v>3.330513028360173</v>
+        <v>6.494888847477548</v>
       </c>
       <c r="G3" t="n">
-        <v>1.67540534359023</v>
+        <v>0.8626238710071714</v>
       </c>
       <c r="H3" t="n">
-        <v>11599.73764398589</v>
+        <v>11549.60431958649</v>
       </c>
       <c r="I3" t="n">
-        <v>1400.207008455474</v>
+        <v>1814.377266938541</v>
       </c>
       <c r="J3" t="n">
         <v>1400</v>
       </c>
       <c r="K3" t="n">
-        <v>11398.38677569813</v>
+        <v>11489.78465608692</v>
       </c>
       <c r="L3" t="n">
-        <v>1400.311143484977</v>
+        <v>1869.413115966614</v>
       </c>
       <c r="M3" t="n">
-        <v>1386.244379488347</v>
+        <v>1396.353440220155</v>
       </c>
     </row>
     <row r="4">
@@ -588,40 +588,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.9826644897248175</v>
+        <v>-0.3384805056011054</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1853928278921927</v>
+        <v>0.940973404155516</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>106.5535871184545</v>
+        <v>81.61786278903227</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7467065974389248</v>
+        <v>8.435134149531351</v>
       </c>
       <c r="G4" t="n">
-        <v>7.79732792358582</v>
+        <v>4.339755946956755</v>
       </c>
       <c r="H4" t="n">
-        <v>5921.815020677005</v>
+        <v>5766.970516147933</v>
       </c>
       <c r="I4" t="n">
-        <v>-2985.249355637709</v>
+        <v>-2352.179688164097</v>
       </c>
       <c r="J4" t="n">
         <v>700</v>
       </c>
       <c r="K4" t="n">
-        <v>5105.384678999153</v>
+        <v>5647.080177661798</v>
       </c>
       <c r="L4" t="n">
-        <v>-2831.218828022905</v>
+        <v>-2018.885397757887</v>
       </c>
       <c r="M4" t="n">
-        <v>402.0578193737633</v>
+        <v>607.7065230313425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement aggressive optimization and multi-algorithm testing
This commit introduces a new aggressive optimization strategy for smoke screen deployment, significantly improving shielding time. It also includes a script for comparing multiple optimization algorithms (PSO, GA, SA, DE) to evaluate their performance.

Co-authored-by: b35etzhangmingyu <b35etzhangmingyu@126.com>
</commit_message>
<xml_diff>
--- a/result2.xlsx
+++ b/result2.xlsx
@@ -502,40 +502,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.9998300494693119</v>
+        <v>0.9883415488938828</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01843562253338214</v>
+        <v>0.1522530220719464</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>95.15925128686945</v>
+        <v>131.2878727802149</v>
       </c>
       <c r="F2" t="n">
-        <v>1.342452273460086</v>
+        <v>0.09844834043078025</v>
       </c>
       <c r="G2" t="n">
-        <v>3.436929578649536</v>
+        <v>0.5352778850482132</v>
       </c>
       <c r="H2" t="n">
-        <v>17672.27495739769</v>
+        <v>17812.77438686003</v>
       </c>
       <c r="I2" t="n">
-        <v>2.355090922428467</v>
+        <v>1.967881454272314</v>
       </c>
       <c r="J2" t="n">
         <v>1800</v>
       </c>
       <c r="K2" t="n">
-        <v>17345.27489524821</v>
+        <v>17882.23057831335</v>
       </c>
       <c r="L2" t="n">
-        <v>8.384565348987348</v>
+        <v>12.66753792648186</v>
       </c>
       <c r="M2" t="n">
-        <v>1742.112917607415</v>
+        <v>1798.595896909107</v>
       </c>
     </row>
     <row r="3">
@@ -545,40 +545,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.7359202316880927</v>
+        <v>0.4884342158042684</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6770682481051257</v>
+        <v>-0.8726007201645374</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>94.23055544662384</v>
+        <v>131.4865712711049</v>
       </c>
       <c r="F3" t="n">
-        <v>6.494888847477548</v>
+        <v>7.05215544366295</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8626238710071714</v>
+        <v>4.852656768007796</v>
       </c>
       <c r="H3" t="n">
-        <v>11549.60431958649</v>
+        <v>12452.90733737711</v>
       </c>
       <c r="I3" t="n">
-        <v>1814.377266938541</v>
+        <v>590.8689932536612</v>
       </c>
       <c r="J3" t="n">
         <v>1400</v>
       </c>
       <c r="K3" t="n">
-        <v>11489.78465608692</v>
+        <v>12764.55728235646</v>
       </c>
       <c r="L3" t="n">
-        <v>1869.413115966614</v>
+        <v>34.09807584274847</v>
       </c>
       <c r="M3" t="n">
-        <v>1396.353440220155</v>
+        <v>1284.601665091496</v>
       </c>
     </row>
     <row r="4">
@@ -588,40 +588,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.3384805056011054</v>
+        <v>-0.7522025263420279</v>
       </c>
       <c r="C4" t="n">
-        <v>0.940973404155516</v>
+        <v>0.6589319838683435</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>81.61786278903227</v>
+        <v>134.6481511774107</v>
       </c>
       <c r="F4" t="n">
-        <v>8.435134149531351</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>4.339755946956755</v>
+        <v>14.44747054007725</v>
       </c>
       <c r="H4" t="n">
-        <v>5766.970516147933</v>
+        <v>3974.346410341367</v>
       </c>
       <c r="I4" t="n">
-        <v>-2352.179688164097</v>
+        <v>-1225.520532409283</v>
       </c>
       <c r="J4" t="n">
         <v>700</v>
       </c>
       <c r="K4" t="n">
-        <v>5647.080177661798</v>
+        <v>2511.067882291625</v>
       </c>
       <c r="L4" t="n">
-        <v>-2018.885397757887</v>
+        <v>56.31645919016046</v>
       </c>
       <c r="M4" t="n">
-        <v>607.7065230313425</v>
+        <v>-322.878449233864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint before follow-up message
Co-authored-by: b35etzhangmingyu <b35etzhangmingyu@126.com>
</commit_message>
<xml_diff>
--- a/result2.xlsx
+++ b/result2.xlsx
@@ -502,40 +502,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9883415488938828</v>
+        <v>0.9925917624702491</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1522530220719464</v>
+        <v>0.1214972965798196</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>131.2878727802149</v>
+        <v>137.4343804234904</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09844834043078025</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5352778850482132</v>
+        <v>0.7304209712983956</v>
       </c>
       <c r="H2" t="n">
-        <v>17812.77438686003</v>
+        <v>17800</v>
       </c>
       <c r="I2" t="n">
-        <v>1.967881454272314</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>1800</v>
       </c>
       <c r="K2" t="n">
-        <v>17882.23057831335</v>
+        <v>17899.64127805775</v>
       </c>
       <c r="L2" t="n">
-        <v>12.66753792648186</v>
+        <v>12.19650048439489</v>
       </c>
       <c r="M2" t="n">
-        <v>1798.595896909107</v>
+        <v>1797.385510745571</v>
       </c>
     </row>
     <row r="3">
@@ -545,40 +545,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4884342158042684</v>
+        <v>0.1382747063625363</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.8726007201645374</v>
+        <v>-0.990393914349414</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>131.4865712711049</v>
+        <v>131.0869067152109</v>
       </c>
       <c r="F3" t="n">
-        <v>7.05215544366295</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>4.852656768007796</v>
+        <v>12</v>
       </c>
       <c r="H3" t="n">
-        <v>12452.90733737711</v>
+        <v>12000</v>
       </c>
       <c r="I3" t="n">
-        <v>590.8689932536612</v>
+        <v>1400</v>
       </c>
       <c r="J3" t="n">
         <v>1400</v>
       </c>
       <c r="K3" t="n">
-        <v>12764.55728235646</v>
+        <v>12217.51204240823</v>
       </c>
       <c r="L3" t="n">
-        <v>34.09807584274847</v>
+        <v>-157.9320959396105</v>
       </c>
       <c r="M3" t="n">
-        <v>1284.601665091496</v>
+        <v>694.328</v>
       </c>
     </row>
     <row r="4">
@@ -588,40 +588,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.7522025263420279</v>
+        <v>-0.9895775472933449</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6589319838683435</v>
+        <v>0.1440009649026271</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>134.6481511774107</v>
+        <v>133.9047798846563</v>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>1.430054792370903</v>
       </c>
       <c r="G4" t="n">
-        <v>14.44747054007725</v>
+        <v>12</v>
       </c>
       <c r="H4" t="n">
-        <v>3974.346410341367</v>
+        <v>5810.504635490525</v>
       </c>
       <c r="I4" t="n">
-        <v>-1225.520532409283</v>
+        <v>-2972.425086433524</v>
       </c>
       <c r="J4" t="n">
         <v>700</v>
       </c>
       <c r="K4" t="n">
-        <v>2511.067882291625</v>
+        <v>4220.394671701165</v>
       </c>
       <c r="L4" t="n">
-        <v>56.31645919016046</v>
+        <v>-2741.036076331951</v>
       </c>
       <c r="M4" t="n">
-        <v>-322.878449233864</v>
+        <v>-5.672000000000025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor: Reduce differential evolution parameters for relay strategy
Co-authored-by: b35etzhangmingyu <b35etzhangmingyu@126.com>
</commit_message>
<xml_diff>
--- a/result2.xlsx
+++ b/result2.xlsx
@@ -502,40 +502,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9925917624702491</v>
+        <v>0.9954777300351043</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1214972965798196</v>
+        <v>0.09499520516402894</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>137.4343804234904</v>
+        <v>140</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.8305645133650037</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7304209712983956</v>
+        <v>0.0357790130941097</v>
       </c>
       <c r="H2" t="n">
-        <v>17800</v>
+        <v>17915.75318669772</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>11.04595048886985</v>
       </c>
       <c r="J2" t="n">
         <v>1800</v>
       </c>
       <c r="K2" t="n">
-        <v>17899.64127805775</v>
+        <v>17920.73959620102</v>
       </c>
       <c r="L2" t="n">
-        <v>12.19650048439489</v>
+        <v>11.52178734539165</v>
       </c>
       <c r="M2" t="n">
-        <v>1797.385510745571</v>
+        <v>1799.993726684819</v>
       </c>
     </row>
     <row r="3">
@@ -545,25 +545,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1382747063625363</v>
+        <v>-1</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.990393914349414</v>
+        <v>-1.224646799147353e-16</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>131.0869067152109</v>
+        <v>111.0842726637019</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>7.339088875530937</v>
       </c>
       <c r="G3" t="n">
-        <v>12</v>
+        <v>7.403303338644778</v>
       </c>
       <c r="H3" t="n">
-        <v>12000</v>
+        <v>11184.74265024738</v>
       </c>
       <c r="I3" t="n">
         <v>1400</v>
@@ -572,13 +572,13 @@
         <v>1400</v>
       </c>
       <c r="K3" t="n">
-        <v>12217.51204240823</v>
+        <v>10362.35208356527</v>
       </c>
       <c r="L3" t="n">
-        <v>-157.9320959396105</v>
+        <v>1400</v>
       </c>
       <c r="M3" t="n">
-        <v>694.328</v>
+        <v>1131.408983962292</v>
       </c>
     </row>
     <row r="4">
@@ -588,40 +588,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.9895775472933449</v>
+        <v>0.2287440578880953</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1440009649026271</v>
+        <v>-0.9734865977407638</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>133.9047798846563</v>
+        <v>70.96236291053069</v>
       </c>
       <c r="F4" t="n">
-        <v>1.430054792370903</v>
+        <v>19.35154722844042</v>
       </c>
       <c r="G4" t="n">
-        <v>12</v>
+        <v>11.13575591775214</v>
       </c>
       <c r="H4" t="n">
-        <v>5810.504635490525</v>
+        <v>6314.118549688141</v>
       </c>
       <c r="I4" t="n">
-        <v>-2972.425086433524</v>
+        <v>-4336.822477691498</v>
       </c>
       <c r="J4" t="n">
         <v>700</v>
       </c>
       <c r="K4" t="n">
-        <v>4220.394671701165</v>
+        <v>6494.876576799513</v>
       </c>
       <c r="L4" t="n">
-        <v>-2741.036076331951</v>
+        <v>-5106.090621535773</v>
       </c>
       <c r="M4" t="n">
-        <v>-5.672000000000025</v>
+        <v>92.31320415728612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>